<commit_message>
Updated script to repo to reflect most recent improvements in TIMESreport tool:
timesreport.gms (replaces TIMESreport/timesreport_DemoS_012.gms)
-expended dimensions of the timesreport parameter by including subsector, service, techgroup, capacityunit, comgroup)
-add sum check for f_in and f_out
-added routine to capture scenario name from vtrun.cmd file.
-added routine to save solver status and solver summary

Scen_Z_TIMESReport.xlsx
- Scen_Z_PRC_GMAP2GDX_WRITE.xlsx has now been included into Scen_Z_TIMESReport.xlsx
- Added SFCmd_bot in order to write description for each commodity and proces set into the raw TIMES-gdx output file so that this information is available to timesreport.gms

SysSettings.xlsx
- Added ~TFM_COMGRP in order to write comgroup into the raw TIMES-gdx output file so that this information is available to timesreport.gms
</commit_message>
<xml_diff>
--- a/Sets-DemoModels.xlsx
+++ b/Sets-DemoModels.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kristoffer\Demo_models\DemoS_012\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kristoffer\DemoS_012_timesreport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53B2AD92-8E72-4B4A-8FB0-D9AAB1341DF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41E15EBF-3D8E-43F6-B664-4A91876615C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="345" yWindow="360" windowWidth="28800" windowHeight="15465" activeTab="1" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="26116" windowHeight="15675" activeTab="2" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
     <sheet name="VEDA_Sets-Proc" sheetId="1" r:id="rId2"/>
+    <sheet name="TIMESreport_Sets-Comm" sheetId="3" r:id="rId3"/>
+    <sheet name="TIMESreport_Sets-Proc" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="187">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -385,14 +387,245 @@
   </si>
   <si>
     <t>ELC*</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>TIMESReport</t>
+  </si>
+  <si>
+    <t>sector</t>
+  </si>
+  <si>
+    <t>service</t>
+  </si>
+  <si>
+    <t>subsector</t>
+  </si>
+  <si>
+    <t>techgroup</t>
+  </si>
+  <si>
+    <t>comgroup</t>
+  </si>
+  <si>
+    <t>Electricity</t>
+  </si>
+  <si>
+    <t>Gas</t>
+  </si>
+  <si>
+    <t>Nuclear</t>
+  </si>
+  <si>
+    <t>Oil</t>
+  </si>
+  <si>
+    <t>Renewable</t>
+  </si>
+  <si>
+    <t>TFM_Csets</t>
+  </si>
+  <si>
+    <t>TR_ELE</t>
+  </si>
+  <si>
+    <t>TR_IND</t>
+  </si>
+  <si>
+    <t>TR_MIN</t>
+  </si>
+  <si>
+    <t>TR_TRD</t>
+  </si>
+  <si>
+    <t>TR_REF</t>
+  </si>
+  <si>
+    <t>TR_AGR</t>
+  </si>
+  <si>
+    <t>TR_COM</t>
+  </si>
+  <si>
+    <t>TR_RES</t>
+  </si>
+  <si>
+    <t>TR_TRA</t>
+  </si>
+  <si>
+    <t>TR_TRM</t>
+  </si>
+  <si>
+    <t>Fossile power plants</t>
+  </si>
+  <si>
+    <t>Nuclear power plants</t>
+  </si>
+  <si>
+    <t>Renewable power plant</t>
+  </si>
+  <si>
+    <t>DMD</t>
+  </si>
+  <si>
+    <t>DIIS</t>
+  </si>
+  <si>
+    <t>Steel service</t>
+  </si>
+  <si>
+    <t>TR_ES_STEEL</t>
+  </si>
+  <si>
+    <t>Space heating</t>
+  </si>
+  <si>
+    <t>Appliances</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>DRSH,DCSH</t>
+  </si>
+  <si>
+    <t>DRAP,DCAP</t>
+  </si>
+  <si>
+    <t>TR_ES_OTH</t>
+  </si>
+  <si>
+    <t>TR_ES_APP</t>
+  </si>
+  <si>
+    <t>TR_ES_SP</t>
+  </si>
+  <si>
+    <t>DIDM1,DROT,DCOT,DAOT</t>
+  </si>
+  <si>
+    <t>Iron&amp;Stell</t>
+  </si>
+  <si>
+    <t>ITIISIN,ITIISIBF,ITIISBOF,IDMIIS</t>
+  </si>
+  <si>
+    <t>TR_STEEL</t>
+  </si>
+  <si>
+    <t>TR_PP_FOSSIL</t>
+  </si>
+  <si>
+    <t>TR_PP_NUCLEAR</t>
+  </si>
+  <si>
+    <t>TR_PP_RENEW</t>
+  </si>
+  <si>
+    <t>Mt-y</t>
+  </si>
+  <si>
+    <t>Million ton a year</t>
+  </si>
+  <si>
+    <t>TFM_Psets</t>
+  </si>
+  <si>
+    <t>EXP*,IMP*,-IMP*Z</t>
+  </si>
+  <si>
+    <t>NRG</t>
+  </si>
+  <si>
+    <t>NRG_OIL</t>
+  </si>
+  <si>
+    <t>NRG_COA</t>
+  </si>
+  <si>
+    <t>Coal</t>
+  </si>
+  <si>
+    <t>TR_TRAPUB</t>
+  </si>
+  <si>
+    <t>Public Transport</t>
+  </si>
+  <si>
+    <t>TCAR*</t>
+  </si>
+  <si>
+    <t>TPUB*</t>
+  </si>
+  <si>
+    <t>Car transport</t>
+  </si>
+  <si>
+    <t>TR_TRACAR</t>
+  </si>
+  <si>
+    <t>TR_ES_TR</t>
+  </si>
+  <si>
+    <t>Transport</t>
+  </si>
+  <si>
+    <t>DTCAR,DTPUB</t>
+  </si>
+  <si>
+    <t>capacityunit</t>
+  </si>
+  <si>
+    <t>PJa</t>
+  </si>
+  <si>
+    <t>PJ annually</t>
+  </si>
+  <si>
+    <t>GW</t>
+  </si>
+  <si>
+    <t>-ITIISIN,-ITIISIBF,-ITIISBOF,-IDMIIS</t>
+  </si>
+  <si>
+    <t>TR_IND,TR_AGR,TR_COM,TR_RES</t>
+  </si>
+  <si>
+    <t>000_Units</t>
+  </si>
+  <si>
+    <t>1000 units</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="\Te\x\t"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -420,7 +653,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -428,17 +661,31 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 5" xfId="1" xr:uid="{B387DD4F-F719-4379-A4FC-680701E911D2}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -751,23 +998,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BD03DB1-DD55-4548-B86E-1F92E13CF8ED}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="65.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="65.86328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="56" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="11" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.86328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.3984375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -793,7 +1040,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
         <v>72</v>
       </c>
@@ -810,7 +1057,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
         <v>21</v>
       </c>
@@ -824,7 +1071,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>76</v>
       </c>
@@ -841,7 +1088,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
         <v>25</v>
       </c>
@@ -855,7 +1102,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
         <v>79</v>
       </c>
@@ -869,7 +1116,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
         <v>81</v>
       </c>
@@ -883,7 +1130,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="C9" t="s">
         <v>83</v>
       </c>
@@ -905,18 +1152,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E06336B7-5D6A-48EE-B122-F085391548AD}">
   <dimension ref="A1:J116"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="6" max="6" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="30.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.73046875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="30.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -948,7 +1195,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" s="1"/>
       <c r="B3" s="1" t="s">
         <v>115</v>
@@ -972,7 +1219,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" s="1"/>
       <c r="B4" s="1" t="s">
         <v>110</v>
@@ -996,7 +1243,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" s="1"/>
       <c r="B5" s="1" t="s">
         <v>53</v>
@@ -1020,7 +1267,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" s="1"/>
       <c r="B6" s="1" t="s">
         <v>87</v>
@@ -1044,7 +1291,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" s="1"/>
       <c r="B7" s="1" t="s">
         <v>90</v>
@@ -1068,7 +1315,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" s="1"/>
       <c r="B8" s="1" t="s">
         <v>93</v>
@@ -1092,7 +1339,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" s="1"/>
       <c r="B9" s="1" t="s">
         <v>96</v>
@@ -1116,7 +1363,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" s="1"/>
       <c r="B10" s="1" t="s">
         <v>111</v>
@@ -1140,7 +1387,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" s="1"/>
       <c r="B11" s="1" t="s">
         <v>106</v>
@@ -1164,7 +1411,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
         <v>109</v>
@@ -1188,7 +1435,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" s="2"/>
       <c r="B13" s="2" t="s">
         <v>11</v>
@@ -1210,7 +1457,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
@@ -1234,7 +1481,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1258,7 +1505,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -1282,7 +1529,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A17" s="2" t="s">
         <v>14</v>
       </c>
@@ -1306,7 +1553,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A18" s="2" t="s">
         <v>14</v>
       </c>
@@ -1330,7 +1577,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>14</v>
       </c>
@@ -1354,7 +1601,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" s="2" t="s">
         <v>14</v>
       </c>
@@ -1378,7 +1625,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A21" s="2" t="s">
         <v>14</v>
       </c>
@@ -1402,7 +1649,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
         <v>14</v>
       </c>
@@ -1426,7 +1673,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A23" s="2" t="s">
         <v>14</v>
       </c>
@@ -1450,7 +1697,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A24" s="2"/>
       <c r="B24" s="2" t="s">
         <v>35</v>
@@ -1472,7 +1719,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>37</v>
       </c>
@@ -1496,7 +1743,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A26" s="2" t="s">
         <v>37</v>
       </c>
@@ -1520,7 +1767,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A27" s="2" t="s">
         <v>37</v>
       </c>
@@ -1544,7 +1791,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A28" s="2" t="s">
         <v>37</v>
       </c>
@@ -1568,7 +1815,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A29" s="2" t="s">
         <v>37</v>
       </c>
@@ -1592,7 +1839,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A30" s="2"/>
       <c r="B30" s="2" t="s">
         <v>48</v>
@@ -1614,7 +1861,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A31" s="2"/>
       <c r="B31" s="2" t="s">
         <v>50</v>
@@ -1636,7 +1883,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>52</v>
       </c>
@@ -1660,7 +1907,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>14</v>
       </c>
@@ -1684,7 +1931,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>14</v>
       </c>
@@ -1708,7 +1955,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A35" s="2" t="s">
         <v>59</v>
       </c>
@@ -1732,7 +1979,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A36" s="2" t="s">
         <v>14</v>
       </c>
@@ -1756,7 +2003,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A37" s="2" t="s">
         <v>14</v>
       </c>
@@ -1780,7 +2027,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A38" s="2" t="s">
         <v>52</v>
       </c>
@@ -1804,7 +2051,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A39" s="2"/>
       <c r="B39" s="2" t="s">
         <v>11</v>
@@ -1826,7 +2073,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A40" s="2" t="s">
         <v>14</v>
       </c>
@@ -1850,7 +2097,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A41" s="2" t="s">
         <v>14</v>
       </c>
@@ -1874,7 +2121,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A42" s="2" t="s">
         <v>14</v>
       </c>
@@ -1898,7 +2145,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>14</v>
       </c>
@@ -1922,7 +2169,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>14</v>
       </c>
@@ -1946,7 +2193,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>14</v>
       </c>
@@ -1970,7 +2217,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>14</v>
       </c>
@@ -1994,7 +2241,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A47" s="2" t="s">
         <v>14</v>
       </c>
@@ -2018,7 +2265,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A48" s="2" t="s">
         <v>14</v>
       </c>
@@ -2042,7 +2289,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A49" s="2" t="s">
         <v>14</v>
       </c>
@@ -2066,7 +2313,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A50" s="2"/>
       <c r="B50" s="2" t="s">
         <v>35</v>
@@ -2088,7 +2335,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>37</v>
       </c>
@@ -2112,7 +2359,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>37</v>
       </c>
@@ -2136,7 +2383,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>37</v>
       </c>
@@ -2160,7 +2407,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A54" s="2" t="s">
         <v>37</v>
       </c>
@@ -2184,7 +2431,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A55" s="2" t="s">
         <v>37</v>
       </c>
@@ -2208,7 +2455,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A56" s="2"/>
       <c r="B56" s="2" t="s">
         <v>48</v>
@@ -2230,7 +2477,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A57" s="2"/>
       <c r="B57" s="2" t="s">
         <v>50</v>
@@ -2252,7 +2499,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A58" s="2" t="s">
         <v>52</v>
       </c>
@@ -2276,7 +2523,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A59" s="2" t="s">
         <v>14</v>
       </c>
@@ -2300,7 +2547,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A60" s="2" t="s">
         <v>14</v>
       </c>
@@ -2324,7 +2571,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
@@ -2348,7 +2595,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A62" s="2" t="s">
         <v>14</v>
       </c>
@@ -2372,7 +2619,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A63" s="2" t="s">
         <v>14</v>
       </c>
@@ -2396,7 +2643,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A64" s="2" t="s">
         <v>52</v>
       </c>
@@ -2420,7 +2667,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A65" s="2"/>
       <c r="B65" s="2" t="s">
         <v>11</v>
@@ -2442,7 +2689,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A66" s="2" t="s">
         <v>14</v>
       </c>
@@ -2466,7 +2713,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A67" s="2" t="s">
         <v>14</v>
       </c>
@@ -2490,7 +2737,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A68" s="2" t="s">
         <v>14</v>
       </c>
@@ -2514,7 +2761,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A69" s="2" t="s">
         <v>14</v>
       </c>
@@ -2538,7 +2785,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A70" s="2" t="s">
         <v>14</v>
       </c>
@@ -2562,7 +2809,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A71" s="2" t="s">
         <v>14</v>
       </c>
@@ -2586,7 +2833,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A72" s="2" t="s">
         <v>14</v>
       </c>
@@ -2610,7 +2857,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A73" s="2" t="s">
         <v>14</v>
       </c>
@@ -2634,7 +2881,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A74" s="2" t="s">
         <v>14</v>
       </c>
@@ -2658,7 +2905,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A75" s="2" t="s">
         <v>14</v>
       </c>
@@ -2682,7 +2929,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A76" s="2"/>
       <c r="B76" s="2" t="s">
         <v>35</v>
@@ -2704,7 +2951,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A77" s="2" t="s">
         <v>37</v>
       </c>
@@ -2728,7 +2975,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A78" s="2" t="s">
         <v>37</v>
       </c>
@@ -2752,7 +2999,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A79" s="2" t="s">
         <v>37</v>
       </c>
@@ -2776,7 +3023,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A80" s="2" t="s">
         <v>37</v>
       </c>
@@ -2800,7 +3047,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A81" s="2" t="s">
         <v>37</v>
       </c>
@@ -2824,7 +3071,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A82" s="2"/>
       <c r="B82" s="2" t="s">
         <v>48</v>
@@ -2846,7 +3093,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A83" s="2"/>
       <c r="B83" s="2" t="s">
         <v>50</v>
@@ -2868,7 +3115,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A84" s="2" t="s">
         <v>52</v>
       </c>
@@ -2892,7 +3139,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A85" s="2" t="s">
         <v>14</v>
       </c>
@@ -2916,7 +3163,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A86" s="2" t="s">
         <v>14</v>
       </c>
@@ -2940,7 +3187,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A87" s="2" t="s">
         <v>59</v>
       </c>
@@ -2964,7 +3211,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A88" s="2" t="s">
         <v>14</v>
       </c>
@@ -2988,7 +3235,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A89" s="2" t="s">
         <v>14</v>
       </c>
@@ -3012,7 +3259,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A90" s="2" t="s">
         <v>52</v>
       </c>
@@ -3036,7 +3283,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A91" s="2"/>
       <c r="B91" s="2" t="s">
         <v>11</v>
@@ -3058,7 +3305,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A92" s="2" t="s">
         <v>14</v>
       </c>
@@ -3082,7 +3329,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A93" s="2" t="s">
         <v>14</v>
       </c>
@@ -3106,7 +3353,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A94" s="2" t="s">
         <v>14</v>
       </c>
@@ -3130,7 +3377,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A95" s="2" t="s">
         <v>14</v>
       </c>
@@ -3154,7 +3401,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A96" s="2" t="s">
         <v>14</v>
       </c>
@@ -3178,7 +3425,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A97" s="2" t="s">
         <v>14</v>
       </c>
@@ -3202,7 +3449,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A98" s="2" t="s">
         <v>14</v>
       </c>
@@ -3226,7 +3473,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A99" s="2" t="s">
         <v>14</v>
       </c>
@@ -3250,7 +3497,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A100" s="2" t="s">
         <v>14</v>
       </c>
@@ -3274,7 +3521,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A101" s="2" t="s">
         <v>14</v>
       </c>
@@ -3298,7 +3545,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A102" s="2"/>
       <c r="B102" s="2" t="s">
         <v>35</v>
@@ -3320,7 +3567,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A103" s="2" t="s">
         <v>37</v>
       </c>
@@ -3344,7 +3591,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A104" s="2" t="s">
         <v>37</v>
       </c>
@@ -3368,7 +3615,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A105" s="2" t="s">
         <v>37</v>
       </c>
@@ -3392,7 +3639,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A106" s="2" t="s">
         <v>37</v>
       </c>
@@ -3416,7 +3663,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A107" s="2" t="s">
         <v>37</v>
       </c>
@@ -3440,7 +3687,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A108" s="2"/>
       <c r="B108" s="2" t="s">
         <v>48</v>
@@ -3462,7 +3709,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A109" s="2"/>
       <c r="B109" s="2" t="s">
         <v>50</v>
@@ -3484,7 +3731,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A110" s="2" t="s">
         <v>52</v>
       </c>
@@ -3508,7 +3755,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A111" s="2" t="s">
         <v>14</v>
       </c>
@@ -3532,7 +3779,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A112" s="2" t="s">
         <v>14</v>
       </c>
@@ -3556,7 +3803,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A113" s="2" t="s">
         <v>59</v>
       </c>
@@ -3580,7 +3827,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A114" s="2" t="s">
         <v>14</v>
       </c>
@@ -3604,7 +3851,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A115" s="2" t="s">
         <v>14</v>
       </c>
@@ -3628,7 +3875,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A116" s="2" t="s">
         <v>52</v>
       </c>
@@ -3655,4 +3902,1046 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92263227-568C-46DF-958A-CFC24654ABFF}">
+  <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+  </sheetPr>
+  <dimension ref="A1:N8"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="5" max="5" width="28.59765625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D3" t="str">
+        <f>L3</f>
+        <v>NRG_ELC</v>
+      </c>
+      <c r="E3" t="str">
+        <f>M3&amp;" [TIMESreport "&amp;N3&amp;"]"</f>
+        <v>Electricity [TIMESreport comgroup]</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" t="s">
+        <v>74</v>
+      </c>
+      <c r="M3" t="s">
+        <v>124</v>
+      </c>
+      <c r="N3" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" t="str">
+        <f>L4</f>
+        <v>NRG_GAS</v>
+      </c>
+      <c r="E4" t="str">
+        <f>M4&amp;" [TIMESreport "&amp;N4&amp;"]"</f>
+        <v>Gas [TIMESreport comgroup]</v>
+      </c>
+      <c r="F4" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" t="s">
+        <v>75</v>
+      </c>
+      <c r="M4" t="s">
+        <v>125</v>
+      </c>
+      <c r="N4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" t="str">
+        <f>L5</f>
+        <v>NRG_NUK</v>
+      </c>
+      <c r="E5" t="str">
+        <f>M5&amp;" [TIMESreport "&amp;N5&amp;"]"</f>
+        <v>Nuclear [TIMESreport comgroup]</v>
+      </c>
+      <c r="F5" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" t="s">
+        <v>78</v>
+      </c>
+      <c r="M5" t="s">
+        <v>126</v>
+      </c>
+      <c r="N5" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D6" t="str">
+        <f>L6</f>
+        <v>NRG_OIL</v>
+      </c>
+      <c r="E6" t="str">
+        <f>M6&amp;" [TIMESreport "&amp;N6&amp;"]"</f>
+        <v>Oil [TIMESreport comgroup]</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6" t="s">
+        <v>167</v>
+      </c>
+      <c r="M6" t="s">
+        <v>127</v>
+      </c>
+      <c r="N6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B7" t="s">
+        <v>81</v>
+      </c>
+      <c r="D7" t="str">
+        <f>L7</f>
+        <v>NRG_RNW</v>
+      </c>
+      <c r="E7" t="str">
+        <f>M7&amp;" [TIMESreport "&amp;N7&amp;"]"</f>
+        <v>Renewable [TIMESreport comgroup]</v>
+      </c>
+      <c r="F7" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" t="s">
+        <v>82</v>
+      </c>
+      <c r="M7" t="s">
+        <v>128</v>
+      </c>
+      <c r="N7" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>166</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="str">
+        <f>L8</f>
+        <v>NRG_COA</v>
+      </c>
+      <c r="E8" t="str">
+        <f>M8&amp;" [TIMESreport "&amp;N8&amp;"]"</f>
+        <v>Coal [TIMESreport comgroup]</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" t="s">
+        <v>168</v>
+      </c>
+      <c r="M8" t="s">
+        <v>169</v>
+      </c>
+      <c r="N8" t="s">
+        <v>123</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F360305-D145-42E6-8DC6-C7E12995353D}">
+  <sheetPr>
+    <tabColor rgb="FF7030A0"/>
+  </sheetPr>
+  <dimension ref="A1:N27"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="27.265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.1328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.3984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.3984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.1328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.9296875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B3" t="s">
+        <v>115</v>
+      </c>
+      <c r="F3" t="str">
+        <f>L3</f>
+        <v>TR_ELE</v>
+      </c>
+      <c r="G3" t="str">
+        <f>M3&amp;" [TIMESreport "&amp;N3&amp;"]"</f>
+        <v>Electricity supply sector [TIMESreport sector]</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" t="s">
+        <v>130</v>
+      </c>
+      <c r="M3" t="s">
+        <v>103</v>
+      </c>
+      <c r="N3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B4" t="s">
+        <v>110</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" ref="F4:F17" si="0">L4</f>
+        <v>TR_IND</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" ref="G4:G17" si="1">M4&amp;" [TIMESreport "&amp;N4&amp;"]"</f>
+        <v>Industry sector [TIMESreport sector]</v>
+      </c>
+      <c r="H4" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" t="s">
+        <v>13</v>
+      </c>
+      <c r="L4" t="s">
+        <v>131</v>
+      </c>
+      <c r="M4" t="s">
+        <v>104</v>
+      </c>
+      <c r="N4" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_MIN</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="1"/>
+        <v>Mining technologies [TIMESreport sector]</v>
+      </c>
+      <c r="H5" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" t="s">
+        <v>132</v>
+      </c>
+      <c r="M5" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B6" t="s">
+        <v>165</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_TRD</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="1"/>
+        <v>Trade technologies [TIMESreport sector]</v>
+      </c>
+      <c r="H6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6" t="s">
+        <v>133</v>
+      </c>
+      <c r="M6" t="s">
+        <v>89</v>
+      </c>
+      <c r="N6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_REF</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="1"/>
+        <v>Refinery  [TIMESreport sector]</v>
+      </c>
+      <c r="H7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" t="s">
+        <v>134</v>
+      </c>
+      <c r="M7" t="s">
+        <v>91</v>
+      </c>
+      <c r="N7" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B8" t="s">
+        <v>93</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_AGR</v>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="1"/>
+        <v>Agriculture sector [TIMESreport sector]</v>
+      </c>
+      <c r="H8" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" t="s">
+        <v>135</v>
+      </c>
+      <c r="M8" t="s">
+        <v>95</v>
+      </c>
+      <c r="N8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_COM</v>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="1"/>
+        <v>Commercial sector [TIMESreport sector]</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9" t="s">
+        <v>136</v>
+      </c>
+      <c r="M9" t="s">
+        <v>100</v>
+      </c>
+      <c r="N9" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B10" t="s">
+        <v>111</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_RES</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="1"/>
+        <v>Residential sector [TIMESreport sector]</v>
+      </c>
+      <c r="H10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I10" t="s">
+        <v>13</v>
+      </c>
+      <c r="L10" t="s">
+        <v>137</v>
+      </c>
+      <c r="M10" t="s">
+        <v>99</v>
+      </c>
+      <c r="N10" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B11" t="s">
+        <v>106</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_TRA</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="1"/>
+        <v>Transport sector [TIMESreport sector]</v>
+      </c>
+      <c r="H11" t="s">
+        <v>13</v>
+      </c>
+      <c r="I11" t="s">
+        <v>13</v>
+      </c>
+      <c r="L11" t="s">
+        <v>138</v>
+      </c>
+      <c r="M11" t="s">
+        <v>102</v>
+      </c>
+      <c r="N11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B12" t="s">
+        <v>109</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_TRM</v>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="1"/>
+        <v>Transmission of electricity and gas [TIMESreport sector]</v>
+      </c>
+      <c r="H12" t="s">
+        <v>13</v>
+      </c>
+      <c r="I12" t="s">
+        <v>13</v>
+      </c>
+      <c r="L12" t="s">
+        <v>139</v>
+      </c>
+      <c r="M12" t="s">
+        <v>108</v>
+      </c>
+      <c r="N12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" t="s">
+        <v>55</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_PP_FOSSIL</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="1"/>
+        <v>Fossile power plants [TIMESreport techgroup]</v>
+      </c>
+      <c r="H13" t="s">
+        <v>13</v>
+      </c>
+      <c r="I13" t="s">
+        <v>13</v>
+      </c>
+      <c r="L13" t="s">
+        <v>159</v>
+      </c>
+      <c r="M13" t="s">
+        <v>140</v>
+      </c>
+      <c r="N13" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_PP_NUCLEAR</v>
+      </c>
+      <c r="G14" t="str">
+        <f t="shared" si="1"/>
+        <v>Nuclear power plants [TIMESreport techgroup]</v>
+      </c>
+      <c r="H14" t="s">
+        <v>13</v>
+      </c>
+      <c r="I14" t="s">
+        <v>13</v>
+      </c>
+      <c r="L14" t="s">
+        <v>160</v>
+      </c>
+      <c r="M14" t="s">
+        <v>141</v>
+      </c>
+      <c r="N14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
+        <v>62</v>
+      </c>
+      <c r="F15" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_PP_RENEW</v>
+      </c>
+      <c r="G15" t="str">
+        <f t="shared" si="1"/>
+        <v>Renewable power plant [TIMESreport techgroup]</v>
+      </c>
+      <c r="H15" t="s">
+        <v>13</v>
+      </c>
+      <c r="I15" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" t="s">
+        <v>161</v>
+      </c>
+      <c r="M15" t="s">
+        <v>142</v>
+      </c>
+      <c r="N15" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>143</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="F16" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_ES_STEEL</v>
+      </c>
+      <c r="G16" t="str">
+        <f t="shared" si="1"/>
+        <v>Steel service [TIMESreport service]</v>
+      </c>
+      <c r="H16" t="s">
+        <v>13</v>
+      </c>
+      <c r="I16" t="s">
+        <v>13</v>
+      </c>
+      <c r="L16" t="s">
+        <v>146</v>
+      </c>
+      <c r="M16" t="s">
+        <v>145</v>
+      </c>
+      <c r="N16" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>143</v>
+      </c>
+      <c r="E17" t="s">
+        <v>155</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" si="0"/>
+        <v>TR_ES_OTH</v>
+      </c>
+      <c r="G17" t="str">
+        <f t="shared" si="1"/>
+        <v>Other [TIMESreport service]</v>
+      </c>
+      <c r="H17" t="s">
+        <v>13</v>
+      </c>
+      <c r="I17" t="s">
+        <v>13</v>
+      </c>
+      <c r="L17" t="s">
+        <v>152</v>
+      </c>
+      <c r="M17" t="s">
+        <v>149</v>
+      </c>
+      <c r="N17" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>143</v>
+      </c>
+      <c r="E18" t="s">
+        <v>150</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" ref="F18:F20" si="2">L18</f>
+        <v>TR_ES_SP</v>
+      </c>
+      <c r="G18" t="str">
+        <f t="shared" ref="G18:G20" si="3">M18&amp;" [TIMESreport "&amp;N18&amp;"]"</f>
+        <v>Space heating [TIMESreport service]</v>
+      </c>
+      <c r="H18" t="s">
+        <v>13</v>
+      </c>
+      <c r="I18" t="s">
+        <v>13</v>
+      </c>
+      <c r="L18" t="s">
+        <v>154</v>
+      </c>
+      <c r="M18" t="s">
+        <v>147</v>
+      </c>
+      <c r="N18" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>143</v>
+      </c>
+      <c r="E19" t="s">
+        <v>151</v>
+      </c>
+      <c r="F19" t="str">
+        <f t="shared" si="2"/>
+        <v>TR_ES_APP</v>
+      </c>
+      <c r="G19" t="str">
+        <f t="shared" si="3"/>
+        <v>Appliances [TIMESreport service]</v>
+      </c>
+      <c r="H19" t="s">
+        <v>13</v>
+      </c>
+      <c r="I19" t="s">
+        <v>13</v>
+      </c>
+      <c r="L19" t="s">
+        <v>153</v>
+      </c>
+      <c r="M19" t="s">
+        <v>148</v>
+      </c>
+      <c r="N19" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>143</v>
+      </c>
+      <c r="E20" t="s">
+        <v>178</v>
+      </c>
+      <c r="F20" t="str">
+        <f t="shared" si="2"/>
+        <v>TR_ES_TR</v>
+      </c>
+      <c r="G20" t="str">
+        <f t="shared" si="3"/>
+        <v>Transport [TIMESreport service]</v>
+      </c>
+      <c r="H20" t="s">
+        <v>13</v>
+      </c>
+      <c r="I20" t="s">
+        <v>13</v>
+      </c>
+      <c r="L20" t="s">
+        <v>176</v>
+      </c>
+      <c r="M20" t="s">
+        <v>177</v>
+      </c>
+      <c r="N20" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B21" t="s">
+        <v>157</v>
+      </c>
+      <c r="F21" t="str">
+        <f t="shared" ref="F21:F22" si="4">L21</f>
+        <v>TR_STEEL</v>
+      </c>
+      <c r="G21" t="str">
+        <f t="shared" ref="G21:G22" si="5">M21&amp;" [TIMESreport "&amp;N21&amp;"]"</f>
+        <v>Iron&amp;Stell [TIMESreport subsector]</v>
+      </c>
+      <c r="H21" t="s">
+        <v>13</v>
+      </c>
+      <c r="I21" t="s">
+        <v>13</v>
+      </c>
+      <c r="L21" t="s">
+        <v>158</v>
+      </c>
+      <c r="M21" t="s">
+        <v>156</v>
+      </c>
+      <c r="N21" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" t="s">
+        <v>172</v>
+      </c>
+      <c r="F22" t="str">
+        <f t="shared" si="4"/>
+        <v>TR_TRAPUB</v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" si="5"/>
+        <v>Public Transport [TIMESreport subsector]</v>
+      </c>
+      <c r="H22" t="s">
+        <v>13</v>
+      </c>
+      <c r="I22" t="s">
+        <v>13</v>
+      </c>
+      <c r="L22" t="s">
+        <v>170</v>
+      </c>
+      <c r="M22" t="s">
+        <v>171</v>
+      </c>
+      <c r="N22" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>143</v>
+      </c>
+      <c r="B23" t="s">
+        <v>173</v>
+      </c>
+      <c r="F23" t="str">
+        <f t="shared" ref="F23" si="6">L23</f>
+        <v>TR_TRACAR</v>
+      </c>
+      <c r="G23" t="str">
+        <f t="shared" ref="G23" si="7">M23&amp;" [TIMESreport "&amp;N23&amp;"]"</f>
+        <v>Car transport [TIMESreport subsector]</v>
+      </c>
+      <c r="H23" t="s">
+        <v>13</v>
+      </c>
+      <c r="I23" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23" t="s">
+        <v>175</v>
+      </c>
+      <c r="M23" t="s">
+        <v>174</v>
+      </c>
+      <c r="N23" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="B24" t="s">
+        <v>157</v>
+      </c>
+      <c r="F24" t="str">
+        <f t="shared" ref="F24:F27" si="8">L24</f>
+        <v>Mt-y</v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" ref="G24:G26" si="9">M24&amp;" [TIMESreport "&amp;N24&amp;"]"</f>
+        <v>Million ton a year [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I24" t="s">
+        <v>13</v>
+      </c>
+      <c r="L24" t="s">
+        <v>162</v>
+      </c>
+      <c r="M24" t="s">
+        <v>163</v>
+      </c>
+      <c r="N24" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>184</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="8"/>
+        <v>PJa</v>
+      </c>
+      <c r="G25" t="str">
+        <f t="shared" si="9"/>
+        <v>PJ annually [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H25" t="s">
+        <v>13</v>
+      </c>
+      <c r="I25" t="s">
+        <v>13</v>
+      </c>
+      <c r="L25" t="s">
+        <v>180</v>
+      </c>
+      <c r="M25" t="s">
+        <v>181</v>
+      </c>
+      <c r="N25" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>130</v>
+      </c>
+      <c r="F26" t="str">
+        <f t="shared" si="8"/>
+        <v>GW</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="9"/>
+        <v>GW [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H26" t="s">
+        <v>13</v>
+      </c>
+      <c r="I26" t="s">
+        <v>13</v>
+      </c>
+      <c r="L26" t="s">
+        <v>182</v>
+      </c>
+      <c r="M26" t="s">
+        <v>182</v>
+      </c>
+      <c r="N26" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>138</v>
+      </c>
+      <c r="F27" t="str">
+        <f t="shared" si="8"/>
+        <v>000_Units</v>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" ref="G27" si="10">M27&amp;" [TIMESreport "&amp;N27&amp;"]"</f>
+        <v>1000 units [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H27" t="s">
+        <v>13</v>
+      </c>
+      <c r="I27" t="s">
+        <v>13</v>
+      </c>
+      <c r="L27" t="s">
+        <v>185</v>
+      </c>
+      <c r="M27" t="s">
+        <v>186</v>
+      </c>
+      <c r="N27" t="s">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
README.md - Improved documentation of how to setup the tool.
timesreport.gms - change sum check from a absolute sum check to a relative sumcheck (more robust to scaled infeasible solutions)
</commit_message>
<xml_diff>
--- a/Sets-DemoModels.xlsx
+++ b/Sets-DemoModels.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda_models\Demo_models\DemoS_012_timesreport-master\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\kristoffer\DemoS_012_timesreport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6341B32A-B8C4-44F1-AD21-F37528D9EA5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7684F212-534F-45FA-80FD-869BDB4EC69B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25060" yWindow="0" windowWidth="13310" windowHeight="21000" activeTab="2" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
+    <workbookView xWindow="4440" yWindow="2970" windowWidth="25395" windowHeight="9195" activeTab="3" xr2:uid="{008F860A-1793-4F78-8899-BE3F7B7A437A}"/>
   </bookViews>
   <sheets>
     <sheet name="VEDA_Sets-Comm" sheetId="2" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="TIMESreport_Sets-Comm" sheetId="3" r:id="rId3"/>
     <sheet name="TIMESreport_Sets-Proc" sheetId="4" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'TIMESreport_Sets-Proc'!$A$2:$N$54</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -38,8 +41,274 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Kristoffer Steen Andersen</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{942B26F1-E7E3-4CB4-BF4E-1633C8218078}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Column A:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> Name of TIMESreport commodity set
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Column B:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> Description of TIMESreport commodity set (used to define labels downstream)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Column C: </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Specifies which TIMESreport dimension the commodity set belongs to
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Columns E-K:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> Standard VEDA filtering approach for each TIMESreport commodity set
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Note:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> When defining sets for a specific TIMESreport dimension, ensure that each commodity belongs to only one element within that dimension. For example, a commodity cannot be part of both NRG_ELC (Electricity) and NRG_GAS (Gas), as this would result in double-counting. If such overlap occurs, timesreport.gms will abort execution.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>User flexibility</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>: The naming conventions, set definitions, and dimension structure are fully customizable by the user. However, modifying the dimensions, e.g., adding additional commodity dimensions to timesreport, requires GAMS programming skills, as changes must be reflected in the timesreport.gms code.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Kristoffer Steen Andersen</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0" shapeId="0" xr:uid="{5FE19655-0160-4772-9D1D-F36D7641D2AF}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Column A</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">: Name of TIMESreport process set
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Column B</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">: Description of TIMESreport process set (used to define labels downstream)
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Column C</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">: Specifies which TIMESreport dimension the process set belongs to
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Columns E-M</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">: Standard VEDA filtering approach for each TIMESreport process set
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Note:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve"> When defining sets for a specific TIMESreport dimension, ensure that each process belongs to only one element within that dimension. For example, a process cannot be part of both SC_AGR (Agriculture sector) and SC_COM (Commercial Sector), as this would result in double-counting. If such overlap occurs, timesreport.gms will abort execution.
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>User flexibility</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>: The naming conventions, set definitions, and dimension structure are fully customizable by the user. However, modifying or adding to additional dimensions (capacityunit, sector, service, subsector, techgroup) requires GAMS programming skills, as changes must be reflected in the timesreport.gms code.</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="947" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1144" uniqueCount="276">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -431,105 +700,18 @@
     <t>TFM_Csets</t>
   </si>
   <si>
-    <t>TR_ELE</t>
-  </si>
-  <si>
-    <t>TR_IND</t>
-  </si>
-  <si>
-    <t>TR_MIN</t>
-  </si>
-  <si>
-    <t>TR_TRD</t>
-  </si>
-  <si>
-    <t>TR_REF</t>
-  </si>
-  <si>
-    <t>TR_AGR</t>
-  </si>
-  <si>
-    <t>TR_COM</t>
-  </si>
-  <si>
-    <t>TR_RES</t>
-  </si>
-  <si>
-    <t>TR_TRA</t>
-  </si>
-  <si>
-    <t>TR_TRM</t>
-  </si>
-  <si>
-    <t>Fossile power plants</t>
-  </si>
-  <si>
-    <t>Nuclear power plants</t>
-  </si>
-  <si>
-    <t>Renewable power plant</t>
-  </si>
-  <si>
     <t>DMD</t>
   </si>
   <si>
     <t>DIIS</t>
   </si>
   <si>
-    <t>Steel service</t>
-  </si>
-  <si>
-    <t>TR_ES_STEEL</t>
-  </si>
-  <si>
-    <t>Space heating</t>
-  </si>
-  <si>
     <t>Appliances</t>
   </si>
   <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>DRSH,DCSH</t>
-  </si>
-  <si>
-    <t>DRAP,DCAP</t>
-  </si>
-  <si>
-    <t>TR_ES_OTH</t>
-  </si>
-  <si>
-    <t>TR_ES_APP</t>
-  </si>
-  <si>
-    <t>TR_ES_SP</t>
-  </si>
-  <si>
-    <t>DIDM1,DROT,DCOT,DAOT</t>
-  </si>
-  <si>
-    <t>Iron&amp;Stell</t>
-  </si>
-  <si>
     <t>ITIISIN,ITIISIBF,ITIISBOF,IDMIIS</t>
   </si>
   <si>
-    <t>TR_STEEL</t>
-  </si>
-  <si>
-    <t>TR_PP_FOSSIL</t>
-  </si>
-  <si>
-    <t>TR_PP_NUCLEAR</t>
-  </si>
-  <si>
-    <t>TR_PP_RENEW</t>
-  </si>
-  <si>
-    <t>Mt-y</t>
-  </si>
-  <si>
     <t>Million ton a year</t>
   </si>
   <si>
@@ -551,33 +733,6 @@
     <t>Coal</t>
   </si>
   <si>
-    <t>TR_TRAPUB</t>
-  </si>
-  <si>
-    <t>Public Transport</t>
-  </si>
-  <si>
-    <t>TCAR*</t>
-  </si>
-  <si>
-    <t>TPUB*</t>
-  </si>
-  <si>
-    <t>Car transport</t>
-  </si>
-  <si>
-    <t>TR_TRACAR</t>
-  </si>
-  <si>
-    <t>TR_ES_TR</t>
-  </si>
-  <si>
-    <t>Transport</t>
-  </si>
-  <si>
-    <t>DTCAR,DTPUB</t>
-  </si>
-  <si>
     <t>capacityunit</t>
   </si>
   <si>
@@ -603,16 +758,396 @@
   </si>
   <si>
     <t>*ELC</t>
+  </si>
+  <si>
+    <t>SS_ELE</t>
+  </si>
+  <si>
+    <t>Power plants</t>
+  </si>
+  <si>
+    <t>SS_CHP</t>
+  </si>
+  <si>
+    <t>Combined heat and power plant</t>
+  </si>
+  <si>
+    <t>SS_HPL</t>
+  </si>
+  <si>
+    <t>Heating plant</t>
+  </si>
+  <si>
+    <t>CHP</t>
+  </si>
+  <si>
+    <t>HPL</t>
+  </si>
+  <si>
+    <t>IISRST</t>
+  </si>
+  <si>
+    <t>Industrial Steel</t>
+  </si>
+  <si>
+    <t>IISIRO</t>
+  </si>
+  <si>
+    <t>Industrial Iron</t>
+  </si>
+  <si>
+    <t>Industrial Ore</t>
+  </si>
+  <si>
+    <t>Industrial Sinter</t>
+  </si>
+  <si>
+    <t>SS_IRO</t>
+  </si>
+  <si>
+    <t>SS_STE</t>
+  </si>
+  <si>
+    <t>SS_ORE</t>
+  </si>
+  <si>
+    <t>SS_SIN</t>
+  </si>
+  <si>
+    <t>IISSIN</t>
+  </si>
+  <si>
+    <t>Industrial IronSteel Demand</t>
+  </si>
+  <si>
+    <t>SS_OIL</t>
+  </si>
+  <si>
+    <t>SS_COA</t>
+  </si>
+  <si>
+    <t>SS_GAS</t>
+  </si>
+  <si>
+    <t>SS_REW</t>
+  </si>
+  <si>
+    <t>MINSOL*,MINWIN*,MINHYD*</t>
+  </si>
+  <si>
+    <t>SS_BIO</t>
+  </si>
+  <si>
+    <t>MINBIO*</t>
+  </si>
+  <si>
+    <t>SS_OXY</t>
+  </si>
+  <si>
+    <t>MININDOXY</t>
+  </si>
+  <si>
+    <t>SS_NUC</t>
+  </si>
+  <si>
+    <t>MINNUC*</t>
+  </si>
+  <si>
+    <t>MINCOA*,IMPCOA*,EXPCOA*</t>
+  </si>
+  <si>
+    <t>MINGAS*,IMPGAS*,EXPGAS*</t>
+  </si>
+  <si>
+    <t>MINOIL*,IMPOIL*,IMPHFO*,IMPGSL*,IMPDSL*,IMPKER*,IMPLPG*,IMPNAP*, IMPPOP*,EXPOIL*,EXPHFO*,EXPGSL*,EXPDSL*,EXPKER*,EXPLPG*,EXPNAP*, EXPPOP*</t>
+  </si>
+  <si>
+    <t>SS_ELC</t>
+  </si>
+  <si>
+    <t>Electricity trade</t>
+  </si>
+  <si>
+    <t>IMPELC*,EXPELC*</t>
+  </si>
+  <si>
+    <t>SS_REF</t>
+  </si>
+  <si>
+    <t>Oil refinary</t>
+  </si>
+  <si>
+    <t>REFEOIL00</t>
+  </si>
+  <si>
+    <t>SS_AGR</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
+    <t>AOTETOT</t>
+  </si>
+  <si>
+    <t>SS_COM</t>
+  </si>
+  <si>
+    <t>Commercial</t>
+  </si>
+  <si>
+    <t>Other demands</t>
+  </si>
+  <si>
+    <t>Room heat</t>
+  </si>
+  <si>
+    <t>Agricultural demand</t>
+  </si>
+  <si>
+    <t>CA*,RA*</t>
+  </si>
+  <si>
+    <t>CO*,RO*</t>
+  </si>
+  <si>
+    <t>CS*,RS*</t>
+  </si>
+  <si>
+    <t>SS_RES</t>
+  </si>
+  <si>
+    <t>Residential</t>
+  </si>
+  <si>
+    <t>SS_TRC</t>
+  </si>
+  <si>
+    <t>Cars</t>
+  </si>
+  <si>
+    <t>SS_TRP</t>
+  </si>
+  <si>
+    <t>Public transport</t>
+  </si>
+  <si>
+    <t>Private transport</t>
+  </si>
+  <si>
+    <t>SS_TRMG</t>
+  </si>
+  <si>
+    <t>SS_TRME</t>
+  </si>
+  <si>
+    <t>Gas transmission</t>
+  </si>
+  <si>
+    <t>Electricity transmission</t>
+  </si>
+  <si>
+    <t>TB_ELC*</t>
+  </si>
+  <si>
+    <t>TU_GAS*</t>
+  </si>
+  <si>
+    <t>Oil supply</t>
+  </si>
+  <si>
+    <t>Coal supply</t>
+  </si>
+  <si>
+    <t>Natural gas supply</t>
+  </si>
+  <si>
+    <t>Renewable energy supply</t>
+  </si>
+  <si>
+    <t>Domestic biomass supply</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oxygen supply </t>
+  </si>
+  <si>
+    <t>Mining nuclear fuel supply</t>
+  </si>
+  <si>
+    <t>TP*</t>
+  </si>
+  <si>
+    <t>TC*</t>
+  </si>
+  <si>
+    <t>TG_OIL</t>
+  </si>
+  <si>
+    <t>TG_BIO</t>
+  </si>
+  <si>
+    <t>TG_NUC</t>
+  </si>
+  <si>
+    <t>TG_REW</t>
+  </si>
+  <si>
+    <t>TG_ELC</t>
+  </si>
+  <si>
+    <t>TG_GAS</t>
+  </si>
+  <si>
+    <t>*BIO*,</t>
+  </si>
+  <si>
+    <t>*NUC*,</t>
+  </si>
+  <si>
+    <t>*SOL*,*WIN*,*HYD*</t>
+  </si>
+  <si>
+    <t>*OIL*,*HFO*,*GSL*,*DSL*,*KER*,*LPG*,*NAP*,*POP*</t>
+  </si>
+  <si>
+    <t>Biomass</t>
+  </si>
+  <si>
+    <t>SC_TRM</t>
+  </si>
+  <si>
+    <t>SC_TRD</t>
+  </si>
+  <si>
+    <t>SC_TRA</t>
+  </si>
+  <si>
+    <t>SC_RES</t>
+  </si>
+  <si>
+    <t>SC_REF</t>
+  </si>
+  <si>
+    <t>SC_MIN</t>
+  </si>
+  <si>
+    <t>SC_IND</t>
+  </si>
+  <si>
+    <t>SC_ELE</t>
+  </si>
+  <si>
+    <t>SC_COM</t>
+  </si>
+  <si>
+    <t>SC_AGR</t>
+  </si>
+  <si>
+    <t>SR_AGR</t>
+  </si>
+  <si>
+    <t>SR_APP</t>
+  </si>
+  <si>
+    <t>SR_OTH</t>
+  </si>
+  <si>
+    <t>SR_RHT</t>
+  </si>
+  <si>
+    <t>SR_TRC</t>
+  </si>
+  <si>
+    <t>SR_TRP</t>
+  </si>
+  <si>
+    <t>TG_COA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coal </t>
+  </si>
+  <si>
+    <t>NRG_BIO</t>
+  </si>
+  <si>
+    <t>R*,-REFEOIL00</t>
+  </si>
+  <si>
+    <t>Mta</t>
+  </si>
+  <si>
+    <t>SR_IRS</t>
+  </si>
+  <si>
+    <t>IISORE,MINIISORE</t>
+  </si>
+  <si>
+    <t>*SOL*,*WIN*,*RNW*,*HYD*,-*SOLID*,-ELCRNW,-RNW</t>
+  </si>
+  <si>
+    <t>*BIO*,*BIO</t>
+  </si>
+  <si>
+    <t>ENV_CO2</t>
+  </si>
+  <si>
+    <t>ENV</t>
+  </si>
+  <si>
+    <t>*CO2</t>
+  </si>
+  <si>
+    <t>IDM1ETOT</t>
+  </si>
+  <si>
+    <t>SS_IND</t>
+  </si>
+  <si>
+    <t>Industry other</t>
+  </si>
+  <si>
+    <t>SR_IND</t>
+  </si>
+  <si>
+    <t>TG_DMD</t>
+  </si>
+  <si>
+    <t>Demand Technology</t>
+  </si>
+  <si>
+    <t>AOTETOT, IDM1ETOT</t>
+  </si>
+  <si>
+    <t>DEM_COM</t>
+  </si>
+  <si>
+    <t>Demand commodity</t>
+  </si>
+  <si>
+    <t>DEM</t>
+  </si>
+  <si>
+    <t>GHG-emission</t>
+  </si>
+  <si>
+    <t>IDMIIS</t>
+  </si>
+  <si>
+    <t>DCOT,DCSH,DAOT,DCAP,DIDM1,DRAP,DROT,DRSH,DTCAR,DTPUB,DIIS</t>
+  </si>
+  <si>
+    <t>Industry Demand</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="3">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="\Te\x\t"/>
+    <numFmt numFmtId="165" formatCode="_([$€]* #,##0.00_);_([$€]* \(#,##0.00\);_([$€]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -635,8 +1170,52 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Courier"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="8"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -655,8 +1234,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="47"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="55"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -665,30 +1256,124 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right/>
-      <top/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment horizontal="left" vertical="center" indent="5"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" applyBorder="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="1" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="23"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="31">
+    <cellStyle name="5x indented GHG Textfiels" xfId="2" xr:uid="{0FB2083B-5C34-47A0-BE95-276FE0B9770C}"/>
+    <cellStyle name="AggOrange_CRFReport-template" xfId="3" xr:uid="{164EDF9C-1345-4285-A590-72E92C418028}"/>
+    <cellStyle name="AggOrange9_CRFReport-template" xfId="4" xr:uid="{7A2E8B0B-A172-405E-B655-610DAC318C60}"/>
+    <cellStyle name="CustomizationCells" xfId="5" xr:uid="{2B02F197-BB62-4282-A0FB-67B255CB7871}"/>
+    <cellStyle name="Euro" xfId="6" xr:uid="{5ABD2E6B-4F5B-4FE2-9054-9798B0268F88}"/>
+    <cellStyle name="InputCells" xfId="7" xr:uid="{59D2DDF5-E990-4D73-8279-FF490C763849}"/>
+    <cellStyle name="Migliaia_tab emissioni" xfId="21" xr:uid="{C9AFF767-3C09-4056-A5C6-5EFD71374C05}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 10" xfId="8" xr:uid="{B22C9995-6E64-4E7A-9C93-5C8C36FC0748}"/>
+    <cellStyle name="Normal 10 2" xfId="19" xr:uid="{3A68CEB6-B267-43CD-A80A-69D8322BAE37}"/>
+    <cellStyle name="Normal 11" xfId="28" xr:uid="{F97EA0D5-487D-4116-9607-3BEB1CA32B6E}"/>
+    <cellStyle name="Normal 12" xfId="23" xr:uid="{8D2A0BBA-0528-4397-900B-6D96E199F205}"/>
+    <cellStyle name="Normal 2" xfId="9" xr:uid="{62134BF4-8887-4886-9159-C353664C4E93}"/>
+    <cellStyle name="Normal 3" xfId="10" xr:uid="{5AA0F7C3-3582-4C87-B283-9B7D69484195}"/>
+    <cellStyle name="Normal 3 2" xfId="27" xr:uid="{6FFD48F4-2248-436D-BAC1-2BF3AFDD0324}"/>
+    <cellStyle name="Normal 3 3" xfId="30" xr:uid="{AAB53E4D-39CB-4C21-A670-E7A674143D64}"/>
+    <cellStyle name="Normal 4" xfId="11" xr:uid="{9B67B6A7-5EA3-456B-A559-EA7CFC7CA5CF}"/>
     <cellStyle name="Normal 5" xfId="1" xr:uid="{B387DD4F-F719-4379-A4FC-680701E911D2}"/>
+    <cellStyle name="Normal 5 2" xfId="26" xr:uid="{EC443464-2DF2-477D-919C-92F1557FA9FE}"/>
+    <cellStyle name="Normal 5 3" xfId="29" xr:uid="{2264DF01-97E2-4FE1-9793-C831AF5424A3}"/>
+    <cellStyle name="Normal 6" xfId="20" xr:uid="{766BC6C5-346A-4CAC-91AF-BBFE8FFB071A}"/>
+    <cellStyle name="Normal 7" xfId="22" xr:uid="{88CD0106-675A-4B14-8A3E-2F4148FD9714}"/>
+    <cellStyle name="Normal 8" xfId="24" xr:uid="{60A7F545-E99D-47AE-A99D-604B7A192563}"/>
+    <cellStyle name="Normal 9" xfId="25" xr:uid="{53D6706E-923C-4BB5-AE55-716FD874A845}"/>
+    <cellStyle name="Normal GHG Numbers (0.00)" xfId="12" xr:uid="{7D199897-9DCA-41DD-A62F-5B1B459715F7}"/>
+    <cellStyle name="Normal GHG Textfiels Bold" xfId="13" xr:uid="{517FA2F6-00A8-4B2F-93B3-CB1F2E12BB06}"/>
+    <cellStyle name="Normal GHG-Shade" xfId="14" xr:uid="{20EC4AB8-9C1E-4B72-8CA6-6F9027FB5200}"/>
+    <cellStyle name="Normale_B2020" xfId="15" xr:uid="{F175AF03-F959-40DB-AB54-7CD7D2C0050D}"/>
+    <cellStyle name="Percent 2" xfId="16" xr:uid="{4BB3658D-C2B8-47C8-A102-E0EF5481323E}"/>
+    <cellStyle name="Standard_Sce_D_Extraction" xfId="17" xr:uid="{99EEC642-FF20-4538-9E84-4B4FC758D80D}"/>
+    <cellStyle name="Обычный_CRF2002 (1)" xfId="18" xr:uid="{0AD22835-B9E3-4CD8-BFAD-DA6B7F27324E}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1163,7 +1848,7 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>164</v>
+        <v>135</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
@@ -3908,1043 +4593,1979 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92263227-568C-46DF-958A-CFC24654ABFF}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92263227-568C-46DF-958A-CFC24654ABFF}">
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="5" max="5" width="28.6328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="31.54296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="28.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>166</v>
+        <v>74</v>
       </c>
       <c r="B3" t="s">
-        <v>187</v>
-      </c>
-      <c r="D3" t="str">
-        <f t="shared" ref="D3:D8" si="0">L3</f>
+        <v>124</v>
+      </c>
+      <c r="C3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E11" si="0">A3</f>
         <v>NRG_ELC</v>
       </c>
-      <c r="E3" t="str">
-        <f t="shared" ref="E3:E8" si="1">M3&amp;" [TIMESreport "&amp;N3&amp;"]"</f>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F11" si="1">B3&amp;" [TIMESreport "&amp;C3&amp;"]"</f>
         <v>Electricity [TIMESreport comgroup]</v>
       </c>
-      <c r="F3" t="s">
-        <v>13</v>
-      </c>
       <c r="G3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L3" t="s">
-        <v>74</v>
-      </c>
-      <c r="M3" t="s">
-        <v>124</v>
-      </c>
-      <c r="N3" t="s">
+        <v>137</v>
+      </c>
+      <c r="H3" t="s">
+        <v>149</v>
+      </c>
+      <c r="J3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>75</v>
+      </c>
+      <c r="B4" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>166</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" t="str">
+      <c r="E4" t="str">
         <f t="shared" si="0"/>
         <v>NRG_GAS</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F4" t="str">
         <f t="shared" si="1"/>
         <v>Gas [TIMESreport comgroup]</v>
       </c>
-      <c r="F4" t="s">
-        <v>13</v>
-      </c>
       <c r="G4" t="s">
-        <v>13</v>
-      </c>
-      <c r="L4" t="s">
-        <v>75</v>
-      </c>
-      <c r="M4" t="s">
-        <v>125</v>
-      </c>
-      <c r="N4" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J4" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>166</v>
-      </c>
-      <c r="B5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" t="str">
+      <c r="E5" t="str">
         <f t="shared" si="0"/>
         <v>NRG_NUK</v>
       </c>
-      <c r="E5" t="str">
+      <c r="F5" t="str">
         <f t="shared" si="1"/>
         <v>Nuclear [TIMESreport comgroup]</v>
       </c>
-      <c r="F5" t="s">
-        <v>13</v>
-      </c>
       <c r="G5" t="s">
-        <v>13</v>
-      </c>
-      <c r="L5" t="s">
-        <v>78</v>
-      </c>
-      <c r="M5" t="s">
-        <v>126</v>
-      </c>
-      <c r="N5" t="s">
+        <v>137</v>
+      </c>
+      <c r="H5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>138</v>
+      </c>
+      <c r="B6" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>166</v>
-      </c>
-      <c r="B6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D6" t="str">
+      <c r="E6" t="str">
         <f t="shared" si="0"/>
         <v>NRG_OIL</v>
       </c>
-      <c r="E6" t="str">
+      <c r="F6" t="str">
         <f t="shared" si="1"/>
         <v>Oil [TIMESreport comgroup]</v>
       </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
       <c r="G6" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6" t="s">
-        <v>167</v>
-      </c>
-      <c r="M6" t="s">
-        <v>127</v>
-      </c>
-      <c r="N6" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" t="s">
+        <v>79</v>
+      </c>
+      <c r="J6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>166</v>
-      </c>
-      <c r="B7" t="s">
-        <v>81</v>
-      </c>
-      <c r="D7" t="str">
+      <c r="E7" t="str">
         <f t="shared" si="0"/>
         <v>NRG_RNW</v>
       </c>
-      <c r="E7" t="str">
+      <c r="F7" t="str">
         <f t="shared" si="1"/>
         <v>Renewable [TIMESreport comgroup]</v>
       </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
       <c r="G7" t="s">
-        <v>13</v>
-      </c>
-      <c r="L7" t="s">
-        <v>82</v>
-      </c>
-      <c r="M7" t="s">
-        <v>128</v>
-      </c>
-      <c r="N7" t="s">
+        <v>137</v>
+      </c>
+      <c r="H7" t="s">
+        <v>257</v>
+      </c>
+      <c r="J7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" t="s">
+        <v>140</v>
+      </c>
+      <c r="C8" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>166</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="str">
+      <c r="E8" t="str">
         <f t="shared" si="0"/>
         <v>NRG_COA</v>
       </c>
-      <c r="E8" t="str">
+      <c r="F8" t="str">
         <f t="shared" si="1"/>
         <v>Coal [TIMESreport comgroup]</v>
       </c>
-      <c r="F8" t="s">
-        <v>13</v>
-      </c>
       <c r="G8" t="s">
-        <v>13</v>
-      </c>
-      <c r="L8" t="s">
-        <v>168</v>
-      </c>
-      <c r="M8" t="s">
-        <v>169</v>
-      </c>
-      <c r="N8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>252</v>
+      </c>
+      <c r="B9" t="s">
+        <v>233</v>
+      </c>
+      <c r="C9" t="s">
         <v>123</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>NRG_BIO</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
+        <v>Biomass [TIMESreport comgroup]</v>
+      </c>
+      <c r="G9" t="s">
+        <v>137</v>
+      </c>
+      <c r="H9" t="s">
+        <v>258</v>
+      </c>
+      <c r="J9" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>259</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C10" t="s">
+        <v>123</v>
+      </c>
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>ENV_CO2</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v>GHG-emission [TIMESreport comgroup]</v>
+      </c>
+      <c r="G10" t="s">
+        <v>260</v>
+      </c>
+      <c r="H10" t="s">
+        <v>261</v>
+      </c>
+      <c r="J10" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>269</v>
+      </c>
+      <c r="B11" t="s">
+        <v>270</v>
+      </c>
+      <c r="C11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E11" t="str">
+        <f t="shared" si="0"/>
+        <v>DEM_COM</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="1"/>
+        <v>Demand commodity [TIMESreport comgroup]</v>
+      </c>
+      <c r="G11" t="s">
+        <v>271</v>
+      </c>
+      <c r="H11" t="s">
+        <v>274</v>
+      </c>
+      <c r="J11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F360305-D145-42E6-8DC6-C7E12995353D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F360305-D145-42E6-8DC6-C7E12995353D}">
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.08984375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.36328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14.08984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="27.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="47.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="143.26953125" customWidth="1"/>
+    <col min="10" max="10" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+      <c r="E1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="H2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="I2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="J2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="K2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="1" t="s">
+      <c r="L2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="1" t="s">
+      <c r="M2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="1" t="s">
+      <c r="N2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="N2" s="3" t="s">
-        <v>118</v>
-      </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>147</v>
+      </c>
       <c r="B3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E36" si="0">A3</f>
+        <v>000_Units</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F36" si="1">B3&amp;" [TIMESreport "&amp;C3&amp;"]"</f>
+        <v>1000 units [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H3" t="s">
+        <v>106</v>
+      </c>
+      <c r="L3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>GW</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="1"/>
+        <v>GW [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H4" t="s">
         <v>115</v>
       </c>
-      <c r="F3" t="str">
-        <f>L3</f>
-        <v>TR_ELE</v>
-      </c>
-      <c r="G3" t="str">
-        <f>M3&amp;" [TIMESreport "&amp;N3&amp;"]"</f>
+      <c r="L4" t="s">
+        <v>13</v>
+      </c>
+      <c r="M4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C5" t="s">
+        <v>141</v>
+      </c>
+      <c r="E5" t="str">
+        <f>A5</f>
+        <v>Mta</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="1"/>
+        <v>Million ton a year [TIMESreport capacityunit]</v>
+      </c>
+      <c r="H5" t="s">
+        <v>133</v>
+      </c>
+      <c r="L5" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>142</v>
+      </c>
+      <c r="B6" t="s">
+        <v>143</v>
+      </c>
+      <c r="C6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>PJa</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="1"/>
+        <v>PJ annually [TIMESreport capacityunit]</v>
+      </c>
+      <c r="G6" t="s">
+        <v>146</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="L6" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_AGR</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="1"/>
+        <v>Agriculture sector [TIMESreport sector]</v>
+      </c>
+      <c r="H7" t="s">
+        <v>93</v>
+      </c>
+      <c r="L7" t="s">
+        <v>13</v>
+      </c>
+      <c r="M7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>242</v>
+      </c>
+      <c r="B8" t="s">
+        <v>100</v>
+      </c>
+      <c r="C8" t="s">
+        <v>119</v>
+      </c>
+      <c r="E8" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_COM</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="1"/>
+        <v>Commercial sector [TIMESreport sector]</v>
+      </c>
+      <c r="H8" t="s">
+        <v>96</v>
+      </c>
+      <c r="L8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>241</v>
+      </c>
+      <c r="B9" t="s">
+        <v>103</v>
+      </c>
+      <c r="C9" t="s">
+        <v>119</v>
+      </c>
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_ELE</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
         <v>Electricity supply sector [TIMESreport sector]</v>
       </c>
-      <c r="H3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I3" t="s">
-        <v>13</v>
-      </c>
-      <c r="L3" t="s">
-        <v>130</v>
-      </c>
-      <c r="M3" t="s">
-        <v>103</v>
-      </c>
-      <c r="N3" t="s">
+      <c r="H9" t="s">
+        <v>115</v>
+      </c>
+      <c r="L9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>240</v>
+      </c>
+      <c r="B10" t="s">
+        <v>104</v>
+      </c>
+      <c r="C10" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B4" t="s">
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_IND</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v>Industry sector [TIMESreport sector]</v>
+      </c>
+      <c r="H10" t="s">
         <v>110</v>
       </c>
-      <c r="F4" t="str">
-        <f t="shared" ref="F4:F17" si="0">L4</f>
-        <v>TR_IND</v>
-      </c>
-      <c r="G4" t="str">
-        <f t="shared" ref="G4:G17" si="1">M4&amp;" [TIMESreport "&amp;N4&amp;"]"</f>
-        <v>Industry sector [TIMESreport sector]</v>
-      </c>
-      <c r="H4" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" t="s">
-        <v>13</v>
-      </c>
-      <c r="L4" t="s">
-        <v>131</v>
-      </c>
-      <c r="M4" t="s">
-        <v>104</v>
-      </c>
-      <c r="N4" t="s">
+      <c r="L10" t="s">
+        <v>13</v>
+      </c>
+      <c r="M10" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>239</v>
+      </c>
+      <c r="B11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C11" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B5" t="s">
-        <v>53</v>
-      </c>
-      <c r="F5" t="str">
+      <c r="E11" t="str">
         <f t="shared" si="0"/>
-        <v>TR_MIN</v>
-      </c>
-      <c r="G5" t="str">
+        <v>SC_MIN</v>
+      </c>
+      <c r="F11" t="str">
         <f t="shared" si="1"/>
         <v>Mining technologies [TIMESreport sector]</v>
       </c>
-      <c r="H5" t="s">
-        <v>13</v>
-      </c>
-      <c r="I5" t="s">
-        <v>13</v>
-      </c>
-      <c r="L5" t="s">
-        <v>132</v>
-      </c>
-      <c r="M5" t="s">
-        <v>86</v>
-      </c>
-      <c r="N5" t="s">
+      <c r="H11" t="s">
+        <v>53</v>
+      </c>
+      <c r="L11" t="s">
+        <v>13</v>
+      </c>
+      <c r="M11" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>238</v>
+      </c>
+      <c r="B12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C12" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B6" t="s">
-        <v>165</v>
-      </c>
-      <c r="F6" t="str">
+      <c r="E12" t="str">
         <f t="shared" si="0"/>
-        <v>TR_TRD</v>
-      </c>
-      <c r="G6" t="str">
+        <v>SC_REF</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="1"/>
+        <v>Refinery  [TIMESreport sector]</v>
+      </c>
+      <c r="H12" t="s">
+        <v>90</v>
+      </c>
+      <c r="L12" t="s">
+        <v>13</v>
+      </c>
+      <c r="M12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>237</v>
+      </c>
+      <c r="B13" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" t="s">
+        <v>119</v>
+      </c>
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_RES</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="1"/>
+        <v>Residential sector [TIMESreport sector]</v>
+      </c>
+      <c r="H13" t="s">
+        <v>111</v>
+      </c>
+      <c r="L13" t="s">
+        <v>13</v>
+      </c>
+      <c r="M13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>236</v>
+      </c>
+      <c r="B14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C14" t="s">
+        <v>119</v>
+      </c>
+      <c r="E14" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_TRA</v>
+      </c>
+      <c r="F14" t="str">
+        <f t="shared" si="1"/>
+        <v>Transport sector [TIMESreport sector]</v>
+      </c>
+      <c r="H14" t="s">
+        <v>106</v>
+      </c>
+      <c r="L14" t="s">
+        <v>13</v>
+      </c>
+      <c r="M14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>235</v>
+      </c>
+      <c r="B15" t="s">
+        <v>89</v>
+      </c>
+      <c r="C15" t="s">
+        <v>119</v>
+      </c>
+      <c r="E15" t="str">
+        <f t="shared" si="0"/>
+        <v>SC_TRD</v>
+      </c>
+      <c r="F15" t="str">
         <f t="shared" si="1"/>
         <v>Trade technologies [TIMESreport sector]</v>
       </c>
-      <c r="H6" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" t="s">
-        <v>13</v>
-      </c>
-      <c r="L6" t="s">
-        <v>133</v>
-      </c>
-      <c r="M6" t="s">
-        <v>89</v>
-      </c>
-      <c r="N6" t="s">
+      <c r="H15" t="s">
+        <v>136</v>
+      </c>
+      <c r="L15" t="s">
+        <v>13</v>
+      </c>
+      <c r="M15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>234</v>
+      </c>
+      <c r="B16" t="s">
+        <v>108</v>
+      </c>
+      <c r="C16" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B7" t="s">
-        <v>90</v>
-      </c>
-      <c r="F7" t="str">
+      <c r="E16" t="str">
         <f t="shared" si="0"/>
-        <v>TR_REF</v>
-      </c>
-      <c r="G7" t="str">
-        <f t="shared" si="1"/>
-        <v>Refinery  [TIMESreport sector]</v>
-      </c>
-      <c r="H7" t="s">
-        <v>13</v>
-      </c>
-      <c r="I7" t="s">
-        <v>13</v>
-      </c>
-      <c r="L7" t="s">
-        <v>134</v>
-      </c>
-      <c r="M7" t="s">
-        <v>91</v>
-      </c>
-      <c r="N7" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
-        <v>93</v>
-      </c>
-      <c r="F8" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_AGR</v>
-      </c>
-      <c r="G8" t="str">
-        <f t="shared" si="1"/>
-        <v>Agriculture sector [TIMESreport sector]</v>
-      </c>
-      <c r="H8" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" t="s">
-        <v>13</v>
-      </c>
-      <c r="L8" t="s">
-        <v>135</v>
-      </c>
-      <c r="M8" t="s">
-        <v>95</v>
-      </c>
-      <c r="N8" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>96</v>
-      </c>
-      <c r="F9" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_COM</v>
-      </c>
-      <c r="G9" t="str">
-        <f t="shared" si="1"/>
-        <v>Commercial sector [TIMESreport sector]</v>
-      </c>
-      <c r="H9" t="s">
-        <v>13</v>
-      </c>
-      <c r="I9" t="s">
-        <v>13</v>
-      </c>
-      <c r="L9" t="s">
-        <v>136</v>
-      </c>
-      <c r="M9" t="s">
-        <v>100</v>
-      </c>
-      <c r="N9" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B10" t="s">
-        <v>111</v>
-      </c>
-      <c r="F10" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_RES</v>
-      </c>
-      <c r="G10" t="str">
-        <f t="shared" si="1"/>
-        <v>Residential sector [TIMESreport sector]</v>
-      </c>
-      <c r="H10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I10" t="s">
-        <v>13</v>
-      </c>
-      <c r="L10" t="s">
-        <v>137</v>
-      </c>
-      <c r="M10" t="s">
-        <v>99</v>
-      </c>
-      <c r="N10" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B11" t="s">
-        <v>106</v>
-      </c>
-      <c r="F11" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_TRA</v>
-      </c>
-      <c r="G11" t="str">
-        <f t="shared" si="1"/>
-        <v>Transport sector [TIMESreport sector]</v>
-      </c>
-      <c r="H11" t="s">
-        <v>13</v>
-      </c>
-      <c r="I11" t="s">
-        <v>13</v>
-      </c>
-      <c r="L11" t="s">
-        <v>138</v>
-      </c>
-      <c r="M11" t="s">
-        <v>102</v>
-      </c>
-      <c r="N11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B12" t="s">
-        <v>109</v>
-      </c>
-      <c r="F12" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_TRM</v>
-      </c>
-      <c r="G12" t="str">
+        <v>SC_TRM</v>
+      </c>
+      <c r="F16" t="str">
         <f t="shared" si="1"/>
         <v>Transmission of electricity and gas [TIMESreport sector]</v>
       </c>
-      <c r="H12" t="s">
-        <v>13</v>
-      </c>
-      <c r="I12" t="s">
-        <v>13</v>
-      </c>
-      <c r="L12" t="s">
-        <v>139</v>
-      </c>
-      <c r="M12" t="s">
-        <v>108</v>
-      </c>
-      <c r="N12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="H16" t="s">
+        <v>109</v>
+      </c>
+      <c r="L16" t="s">
+        <v>13</v>
+      </c>
+      <c r="M16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>244</v>
+      </c>
+      <c r="B17" t="s">
+        <v>197</v>
+      </c>
+      <c r="C17" t="s">
+        <v>120</v>
+      </c>
+      <c r="E17" t="str">
+        <f t="shared" ref="E17" si="2">A17</f>
+        <v>SR_AGR</v>
+      </c>
+      <c r="F17" t="str">
+        <f t="shared" ref="F17" si="3">B17&amp;" [TIMESreport "&amp;C17&amp;"]"</f>
+        <v>Agricultural demand [TIMESreport service]</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="L17" t="s">
+        <v>13</v>
+      </c>
+      <c r="M17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>245</v>
+      </c>
+      <c r="B18" t="s">
+        <v>132</v>
+      </c>
+      <c r="C18" t="s">
+        <v>120</v>
+      </c>
+      <c r="E18" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_APP</v>
+      </c>
+      <c r="F18" t="str">
+        <f t="shared" si="1"/>
+        <v>Appliances [TIMESreport service]</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="L18" t="s">
+        <v>13</v>
+      </c>
+      <c r="M18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>255</v>
+      </c>
+      <c r="B19" t="s">
+        <v>169</v>
+      </c>
+      <c r="C19" t="s">
+        <v>120</v>
+      </c>
+      <c r="E19" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_IRS</v>
+      </c>
+      <c r="F19" t="str">
+        <f t="shared" si="1"/>
+        <v>Industrial IronSteel Demand [TIMESreport service]</v>
+      </c>
+      <c r="G19" t="s">
+        <v>130</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>273</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="L19" t="s">
+        <v>13</v>
+      </c>
+      <c r="M19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>265</v>
+      </c>
+      <c r="B20" t="s">
+        <v>275</v>
+      </c>
+      <c r="C20" t="s">
+        <v>120</v>
+      </c>
+      <c r="E20" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_IND</v>
+      </c>
+      <c r="F20" t="str">
+        <f t="shared" si="1"/>
+        <v>Industry Demand [TIMESreport service]</v>
+      </c>
+      <c r="G20" t="s">
+        <v>130</v>
+      </c>
+      <c r="H20" t="s">
+        <v>262</v>
+      </c>
+      <c r="K20" s="5"/>
+      <c r="L20" t="s">
+        <v>13</v>
+      </c>
+      <c r="M20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>246</v>
+      </c>
+      <c r="B21" t="s">
+        <v>195</v>
+      </c>
+      <c r="C21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_OTH</v>
+      </c>
+      <c r="F21" t="str">
+        <f t="shared" si="1"/>
+        <v>Other demands [TIMESreport service]</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="L21" t="s">
+        <v>13</v>
+      </c>
+      <c r="M21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>247</v>
+      </c>
+      <c r="B22" t="s">
+        <v>196</v>
+      </c>
+      <c r="C22" t="s">
+        <v>120</v>
+      </c>
+      <c r="E22" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_RHT</v>
+      </c>
+      <c r="F22" t="str">
+        <f t="shared" si="1"/>
+        <v>Room heat [TIMESreport service]</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="L22" t="s">
+        <v>13</v>
+      </c>
+      <c r="M22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>248</v>
+      </c>
+      <c r="B23" t="s">
+        <v>204</v>
+      </c>
+      <c r="C23" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_TRC</v>
+      </c>
+      <c r="F23" t="str">
+        <f t="shared" si="1"/>
+        <v>Cars [TIMESreport service]</v>
+      </c>
+      <c r="G23" t="s">
+        <v>130</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="L23" t="s">
+        <v>13</v>
+      </c>
+      <c r="M23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>249</v>
+      </c>
+      <c r="B24" t="s">
+        <v>206</v>
+      </c>
+      <c r="C24" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" t="str">
+        <f t="shared" si="0"/>
+        <v>SR_TRP</v>
+      </c>
+      <c r="F24" t="str">
+        <f t="shared" si="1"/>
+        <v>Public transport [TIMESreport service]</v>
+      </c>
+      <c r="G24" t="s">
+        <v>130</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="L24" t="s">
+        <v>13</v>
+      </c>
+      <c r="M24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>190</v>
+      </c>
+      <c r="B25" t="s">
+        <v>191</v>
+      </c>
+      <c r="C25" t="s">
+        <v>121</v>
+      </c>
+      <c r="E25" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_AGR</v>
+      </c>
+      <c r="F25" t="str">
+        <f t="shared" si="1"/>
+        <v>Agriculture [TIMESreport subsector]</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="K25" s="5"/>
+      <c r="L25" t="s">
+        <v>13</v>
+      </c>
+      <c r="M25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>175</v>
+      </c>
+      <c r="B26" t="s">
+        <v>218</v>
+      </c>
+      <c r="C26" t="s">
+        <v>121</v>
+      </c>
+      <c r="E26" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_BIO</v>
+      </c>
+      <c r="F26" t="str">
+        <f t="shared" si="1"/>
+        <v>Domestic biomass supply [TIMESreport subsector]</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="K26" s="5"/>
+      <c r="L26" t="s">
+        <v>13</v>
+      </c>
+      <c r="M26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>152</v>
+      </c>
+      <c r="B27" t="s">
+        <v>153</v>
+      </c>
+      <c r="C27" t="s">
+        <v>121</v>
+      </c>
+      <c r="E27" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_CHP</v>
+      </c>
+      <c r="F27" t="str">
+        <f t="shared" si="1"/>
+        <v>Combined heat and power plant [TIMESreport subsector]</v>
+      </c>
+      <c r="G27" t="s">
+        <v>156</v>
+      </c>
+      <c r="H27" t="s">
+        <v>115</v>
+      </c>
+      <c r="L27" t="s">
+        <v>13</v>
+      </c>
+      <c r="M27" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>171</v>
+      </c>
+      <c r="B28" t="s">
+        <v>215</v>
+      </c>
+      <c r="C28" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_COA</v>
+      </c>
+      <c r="F28" t="str">
+        <f t="shared" si="1"/>
+        <v>Coal supply [TIMESreport subsector]</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="K28" s="5"/>
+      <c r="L28" t="s">
+        <v>13</v>
+      </c>
+      <c r="M28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>193</v>
+      </c>
+      <c r="B29" t="s">
+        <v>194</v>
+      </c>
+      <c r="C29" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_COM</v>
+      </c>
+      <c r="F29" t="str">
+        <f t="shared" si="1"/>
+        <v>Commercial [TIMESreport subsector]</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="L29" t="s">
+        <v>13</v>
+      </c>
+      <c r="M29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>184</v>
+      </c>
+      <c r="B30" t="s">
+        <v>185</v>
+      </c>
+      <c r="C30" t="s">
+        <v>121</v>
+      </c>
+      <c r="E30" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_ELC</v>
+      </c>
+      <c r="F30" t="str">
+        <f t="shared" si="1"/>
+        <v>Electricity trade [TIMESreport subsector]</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="K30" s="5"/>
+      <c r="L30" t="s">
+        <v>13</v>
+      </c>
+      <c r="M30" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>150</v>
+      </c>
+      <c r="B31" t="s">
+        <v>151</v>
+      </c>
+      <c r="C31" t="s">
+        <v>121</v>
+      </c>
+      <c r="E31" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_ELE</v>
+      </c>
+      <c r="F31" t="str">
+        <f t="shared" si="1"/>
+        <v>Power plants [TIMESreport subsector]</v>
+      </c>
+      <c r="G31" t="s">
         <v>14</v>
       </c>
-      <c r="D13" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" t="str">
+      <c r="H31" t="s">
+        <v>115</v>
+      </c>
+      <c r="L31" t="s">
+        <v>13</v>
+      </c>
+      <c r="M31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>172</v>
+      </c>
+      <c r="B32" t="s">
+        <v>216</v>
+      </c>
+      <c r="C32" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" t="str">
         <f t="shared" si="0"/>
-        <v>TR_PP_FOSSIL</v>
-      </c>
-      <c r="G13" t="str">
+        <v>SS_GAS</v>
+      </c>
+      <c r="F32" t="str">
         <f t="shared" si="1"/>
-        <v>Fossile power plants [TIMESreport techgroup]</v>
-      </c>
-      <c r="H13" t="s">
-        <v>13</v>
-      </c>
-      <c r="I13" t="s">
-        <v>13</v>
-      </c>
-      <c r="L13" t="s">
+        <v>Natural gas supply [TIMESreport subsector]</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="K32" s="5"/>
+      <c r="L32" t="s">
+        <v>13</v>
+      </c>
+      <c r="M32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>154</v>
+      </c>
+      <c r="B33" t="s">
+        <v>155</v>
+      </c>
+      <c r="C33" t="s">
+        <v>121</v>
+      </c>
+      <c r="E33" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_HPL</v>
+      </c>
+      <c r="F33" t="str">
+        <f t="shared" si="1"/>
+        <v>Heating plant [TIMESreport subsector]</v>
+      </c>
+      <c r="G33" t="s">
+        <v>157</v>
+      </c>
+      <c r="H33" t="s">
+        <v>115</v>
+      </c>
+      <c r="L33" t="s">
+        <v>13</v>
+      </c>
+      <c r="M33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>164</v>
+      </c>
+      <c r="B34" t="s">
+        <v>161</v>
+      </c>
+      <c r="C34" t="s">
+        <v>121</v>
+      </c>
+      <c r="E34" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_IRO</v>
+      </c>
+      <c r="F34" t="str">
+        <f t="shared" si="1"/>
+        <v>Industrial Iron [TIMESreport subsector]</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="L34" t="s">
+        <v>13</v>
+      </c>
+      <c r="M34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>263</v>
+      </c>
+      <c r="B35" t="s">
+        <v>264</v>
+      </c>
+      <c r="C35" t="s">
+        <v>121</v>
+      </c>
+      <c r="E35" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_IND</v>
+      </c>
+      <c r="F35" t="str">
+        <f t="shared" si="1"/>
+        <v>Industry other [TIMESreport subsector]</v>
+      </c>
+      <c r="H35" t="s">
+        <v>262</v>
+      </c>
+      <c r="L35" t="s">
+        <v>13</v>
+      </c>
+      <c r="M35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>179</v>
+      </c>
+      <c r="B36" t="s">
+        <v>220</v>
+      </c>
+      <c r="C36" t="s">
+        <v>121</v>
+      </c>
+      <c r="E36" t="str">
+        <f t="shared" si="0"/>
+        <v>SS_NUC</v>
+      </c>
+      <c r="F36" t="str">
+        <f t="shared" si="1"/>
+        <v>Mining nuclear fuel supply [TIMESreport subsector]</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="K36" s="5"/>
+      <c r="L36" t="s">
+        <v>13</v>
+      </c>
+      <c r="M36" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>170</v>
+      </c>
+      <c r="B37" t="s">
+        <v>214</v>
+      </c>
+      <c r="C37" t="s">
+        <v>121</v>
+      </c>
+      <c r="E37" t="str">
+        <f t="shared" ref="E37:E56" si="4">A37</f>
+        <v>SS_OIL</v>
+      </c>
+      <c r="F37" t="str">
+        <f t="shared" ref="F37:F55" si="5">B37&amp;" [TIMESreport "&amp;C37&amp;"]"</f>
+        <v>Oil supply [TIMESreport subsector]</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="K37" s="5"/>
+      <c r="L37" t="s">
+        <v>13</v>
+      </c>
+      <c r="M37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>166</v>
+      </c>
+      <c r="B38" t="s">
+        <v>162</v>
+      </c>
+      <c r="C38" t="s">
+        <v>121</v>
+      </c>
+      <c r="E38" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_ORE</v>
+      </c>
+      <c r="F38" t="str">
+        <f t="shared" si="5"/>
+        <v>Industrial Ore [TIMESreport subsector]</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="L38" t="s">
+        <v>13</v>
+      </c>
+      <c r="M38" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>177</v>
+      </c>
+      <c r="B39" t="s">
+        <v>219</v>
+      </c>
+      <c r="C39" t="s">
+        <v>121</v>
+      </c>
+      <c r="E39" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_OXY</v>
+      </c>
+      <c r="F39" t="str">
+        <f t="shared" si="5"/>
+        <v>Oxygen supply  [TIMESreport subsector]</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="K39" s="5"/>
+      <c r="L39" t="s">
+        <v>13</v>
+      </c>
+      <c r="M39" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>187</v>
+      </c>
+      <c r="B40" t="s">
+        <v>188</v>
+      </c>
+      <c r="C40" t="s">
+        <v>121</v>
+      </c>
+      <c r="E40" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_REF</v>
+      </c>
+      <c r="F40" t="str">
+        <f t="shared" si="5"/>
+        <v>Oil refinary [TIMESreport subsector]</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="K40" s="5"/>
+      <c r="L40" t="s">
+        <v>13</v>
+      </c>
+      <c r="M40" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>201</v>
+      </c>
+      <c r="B41" t="s">
+        <v>202</v>
+      </c>
+      <c r="C41" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_RES</v>
+      </c>
+      <c r="F41" t="str">
+        <f t="shared" si="5"/>
+        <v>Residential [TIMESreport subsector]</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="L41" t="s">
+        <v>13</v>
+      </c>
+      <c r="M41" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>173</v>
+      </c>
+      <c r="B42" t="s">
+        <v>217</v>
+      </c>
+      <c r="C42" t="s">
+        <v>121</v>
+      </c>
+      <c r="E42" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_REW</v>
+      </c>
+      <c r="F42" t="str">
+        <f t="shared" si="5"/>
+        <v>Renewable energy supply [TIMESreport subsector]</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="K42" s="5"/>
+      <c r="L42" t="s">
+        <v>13</v>
+      </c>
+      <c r="M42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>167</v>
+      </c>
+      <c r="B43" t="s">
+        <v>163</v>
+      </c>
+      <c r="C43" t="s">
+        <v>121</v>
+      </c>
+      <c r="E43" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_SIN</v>
+      </c>
+      <c r="F43" t="str">
+        <f t="shared" si="5"/>
+        <v>Industrial Sinter [TIMESreport subsector]</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="L43" t="s">
+        <v>13</v>
+      </c>
+      <c r="M43" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>165</v>
+      </c>
+      <c r="B44" t="s">
         <v>159</v>
       </c>
-      <c r="M13" t="s">
-        <v>140</v>
-      </c>
-      <c r="N13" t="s">
+      <c r="C44" t="s">
+        <v>121</v>
+      </c>
+      <c r="E44" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_STE</v>
+      </c>
+      <c r="F44" t="str">
+        <f t="shared" si="5"/>
+        <v>Industrial Steel [TIMESreport subsector]</v>
+      </c>
+      <c r="H44" t="s">
+        <v>158</v>
+      </c>
+      <c r="L44" t="s">
+        <v>13</v>
+      </c>
+      <c r="M44" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>203</v>
+      </c>
+      <c r="B45" t="s">
+        <v>207</v>
+      </c>
+      <c r="C45" t="s">
+        <v>121</v>
+      </c>
+      <c r="E45" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_TRC</v>
+      </c>
+      <c r="F45" t="str">
+        <f t="shared" si="5"/>
+        <v>Private transport [TIMESreport subsector]</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="L45" t="s">
+        <v>13</v>
+      </c>
+      <c r="M45" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
+        <v>209</v>
+      </c>
+      <c r="B46" t="s">
+        <v>211</v>
+      </c>
+      <c r="C46" t="s">
+        <v>121</v>
+      </c>
+      <c r="E46" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_TRME</v>
+      </c>
+      <c r="F46" t="str">
+        <f t="shared" si="5"/>
+        <v>Electricity transmission [TIMESreport subsector]</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="L46" t="s">
+        <v>13</v>
+      </c>
+      <c r="M46" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>208</v>
+      </c>
+      <c r="B47" t="s">
+        <v>210</v>
+      </c>
+      <c r="C47" t="s">
+        <v>121</v>
+      </c>
+      <c r="E47" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_TRMG</v>
+      </c>
+      <c r="F47" t="str">
+        <f t="shared" si="5"/>
+        <v>Gas transmission [TIMESreport subsector]</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="L47" t="s">
+        <v>13</v>
+      </c>
+      <c r="M47" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>205</v>
+      </c>
+      <c r="B48" t="s">
+        <v>206</v>
+      </c>
+      <c r="C48" t="s">
+        <v>121</v>
+      </c>
+      <c r="E48" t="str">
+        <f t="shared" si="4"/>
+        <v>SS_TRP</v>
+      </c>
+      <c r="F48" t="str">
+        <f t="shared" si="5"/>
+        <v>Public transport [TIMESreport subsector]</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="L48" t="s">
+        <v>13</v>
+      </c>
+      <c r="M48" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
+        <v>224</v>
+      </c>
+      <c r="B49" t="s">
+        <v>233</v>
+      </c>
+      <c r="C49" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="E49" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_BIO</v>
+      </c>
+      <c r="F49" t="str">
+        <f t="shared" si="5"/>
+        <v>Biomass [TIMESreport techgroup]</v>
+      </c>
+      <c r="H49" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="L49" t="s">
+        <v>13</v>
+      </c>
+      <c r="M49" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
+        <v>227</v>
+      </c>
+      <c r="B50" t="s">
+        <v>124</v>
+      </c>
+      <c r="C50" t="s">
+        <v>122</v>
+      </c>
+      <c r="E50" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_ELC</v>
+      </c>
+      <c r="F50" t="str">
+        <f t="shared" si="5"/>
+        <v>Electricity [TIMESreport techgroup]</v>
+      </c>
+      <c r="H50" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="J50" t="s">
+        <v>149</v>
+      </c>
+      <c r="L50" t="s">
+        <v>13</v>
+      </c>
+      <c r="M50" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
+        <v>228</v>
+      </c>
+      <c r="B51" t="s">
+        <v>125</v>
+      </c>
+      <c r="C51" t="s">
+        <v>122</v>
+      </c>
+      <c r="E51" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_GAS</v>
+      </c>
+      <c r="F51" t="str">
+        <f t="shared" si="5"/>
+        <v>Gas [TIMESreport techgroup]</v>
+      </c>
+      <c r="H51" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="L51" t="s">
+        <v>13</v>
+      </c>
+      <c r="M51" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
+        <v>225</v>
+      </c>
+      <c r="B52" t="s">
+        <v>126</v>
+      </c>
+      <c r="C52" t="s">
+        <v>122</v>
+      </c>
+      <c r="E52" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_NUC</v>
+      </c>
+      <c r="F52" t="str">
+        <f t="shared" si="5"/>
+        <v>Nuclear [TIMESreport techgroup]</v>
+      </c>
+      <c r="H52" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="J52" t="s">
         <v>57</v>
       </c>
-      <c r="F14" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_PP_NUCLEAR</v>
-      </c>
-      <c r="G14" t="str">
-        <f t="shared" si="1"/>
-        <v>Nuclear power plants [TIMESreport techgroup]</v>
-      </c>
-      <c r="H14" t="s">
-        <v>13</v>
-      </c>
-      <c r="I14" t="s">
-        <v>13</v>
-      </c>
-      <c r="L14" t="s">
-        <v>160</v>
-      </c>
-      <c r="M14" t="s">
-        <v>141</v>
-      </c>
-      <c r="N14" t="s">
+      <c r="L52" t="s">
+        <v>13</v>
+      </c>
+      <c r="M52" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
+        <v>223</v>
+      </c>
+      <c r="B53" t="s">
+        <v>127</v>
+      </c>
+      <c r="C53" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" t="s">
-        <v>62</v>
-      </c>
-      <c r="F15" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_PP_RENEW</v>
-      </c>
-      <c r="G15" t="str">
-        <f t="shared" si="1"/>
-        <v>Renewable power plant [TIMESreport techgroup]</v>
-      </c>
-      <c r="H15" t="s">
-        <v>13</v>
-      </c>
-      <c r="I15" t="s">
-        <v>13</v>
-      </c>
-      <c r="L15" t="s">
-        <v>161</v>
-      </c>
-      <c r="M15" t="s">
-        <v>142</v>
-      </c>
-      <c r="N15" t="s">
+      <c r="E53" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_OIL</v>
+      </c>
+      <c r="F53" t="str">
+        <f t="shared" si="5"/>
+        <v>Oil [TIMESreport techgroup]</v>
+      </c>
+      <c r="H53" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="J53" s="5"/>
+      <c r="L53" t="s">
+        <v>13</v>
+      </c>
+      <c r="M53" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="54" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
+        <v>226</v>
+      </c>
+      <c r="B54" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>143</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="F16" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_ES_STEEL</v>
-      </c>
-      <c r="G16" t="str">
-        <f t="shared" si="1"/>
-        <v>Steel service [TIMESreport service]</v>
-      </c>
-      <c r="H16" t="s">
-        <v>13</v>
-      </c>
-      <c r="I16" t="s">
-        <v>13</v>
-      </c>
-      <c r="L16" t="s">
-        <v>146</v>
-      </c>
-      <c r="M16" t="s">
-        <v>145</v>
-      </c>
-      <c r="N16" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>143</v>
-      </c>
-      <c r="E17" t="s">
-        <v>155</v>
-      </c>
-      <c r="F17" t="str">
-        <f t="shared" si="0"/>
-        <v>TR_ES_OTH</v>
-      </c>
-      <c r="G17" t="str">
-        <f t="shared" si="1"/>
-        <v>Other [TIMESreport service]</v>
-      </c>
-      <c r="H17" t="s">
-        <v>13</v>
-      </c>
-      <c r="I17" t="s">
-        <v>13</v>
-      </c>
-      <c r="L17" t="s">
-        <v>152</v>
-      </c>
-      <c r="M17" t="s">
-        <v>149</v>
-      </c>
-      <c r="N17" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>143</v>
-      </c>
-      <c r="E18" t="s">
-        <v>150</v>
-      </c>
-      <c r="F18" t="str">
-        <f t="shared" ref="F18:F20" si="2">L18</f>
-        <v>TR_ES_SP</v>
-      </c>
-      <c r="G18" t="str">
-        <f t="shared" ref="G18:G20" si="3">M18&amp;" [TIMESreport "&amp;N18&amp;"]"</f>
-        <v>Space heating [TIMESreport service]</v>
-      </c>
-      <c r="H18" t="s">
-        <v>13</v>
-      </c>
-      <c r="I18" t="s">
-        <v>13</v>
-      </c>
-      <c r="L18" t="s">
-        <v>154</v>
-      </c>
-      <c r="M18" t="s">
-        <v>147</v>
-      </c>
-      <c r="N18" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>143</v>
-      </c>
-      <c r="E19" t="s">
-        <v>151</v>
-      </c>
-      <c r="F19" t="str">
-        <f t="shared" si="2"/>
-        <v>TR_ES_APP</v>
-      </c>
-      <c r="G19" t="str">
-        <f t="shared" si="3"/>
-        <v>Appliances [TIMESreport service]</v>
-      </c>
-      <c r="H19" t="s">
-        <v>13</v>
-      </c>
-      <c r="I19" t="s">
-        <v>13</v>
-      </c>
-      <c r="L19" t="s">
-        <v>153</v>
-      </c>
-      <c r="M19" t="s">
-        <v>148</v>
-      </c>
-      <c r="N19" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>143</v>
-      </c>
-      <c r="E20" t="s">
-        <v>178</v>
-      </c>
-      <c r="F20" t="str">
-        <f t="shared" si="2"/>
-        <v>TR_ES_TR</v>
-      </c>
-      <c r="G20" t="str">
-        <f t="shared" si="3"/>
-        <v>Transport [TIMESreport service]</v>
-      </c>
-      <c r="H20" t="s">
-        <v>13</v>
-      </c>
-      <c r="I20" t="s">
-        <v>13</v>
-      </c>
-      <c r="L20" t="s">
-        <v>176</v>
-      </c>
-      <c r="M20" t="s">
-        <v>177</v>
-      </c>
-      <c r="N20" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B21" t="s">
-        <v>157</v>
-      </c>
-      <c r="F21" t="str">
-        <f t="shared" ref="F21:F22" si="4">L21</f>
-        <v>TR_STEEL</v>
-      </c>
-      <c r="G21" t="str">
-        <f t="shared" ref="G21:G22" si="5">M21&amp;" [TIMESreport "&amp;N21&amp;"]"</f>
-        <v>Iron&amp;Stell [TIMESreport subsector]</v>
-      </c>
-      <c r="H21" t="s">
-        <v>13</v>
-      </c>
-      <c r="I21" t="s">
-        <v>13</v>
-      </c>
-      <c r="L21" t="s">
-        <v>158</v>
-      </c>
-      <c r="M21" t="s">
-        <v>156</v>
-      </c>
-      <c r="N21" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>143</v>
-      </c>
-      <c r="B22" t="s">
-        <v>172</v>
-      </c>
-      <c r="F22" t="str">
+      <c r="E54" t="str">
         <f t="shared" si="4"/>
-        <v>TR_TRAPUB</v>
-      </c>
-      <c r="G22" t="str">
+        <v>TG_REW</v>
+      </c>
+      <c r="F54" t="str">
         <f t="shared" si="5"/>
-        <v>Public Transport [TIMESreport subsector]</v>
-      </c>
-      <c r="H22" t="s">
-        <v>13</v>
-      </c>
-      <c r="I22" t="s">
-        <v>13</v>
-      </c>
-      <c r="L22" t="s">
-        <v>170</v>
-      </c>
-      <c r="M22" t="s">
-        <v>171</v>
-      </c>
-      <c r="N22" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>143</v>
-      </c>
-      <c r="B23" t="s">
-        <v>173</v>
-      </c>
-      <c r="F23" t="str">
-        <f t="shared" ref="F23" si="6">L23</f>
-        <v>TR_TRACAR</v>
-      </c>
-      <c r="G23" t="str">
-        <f t="shared" ref="G23" si="7">M23&amp;" [TIMESreport "&amp;N23&amp;"]"</f>
-        <v>Car transport [TIMESreport subsector]</v>
-      </c>
-      <c r="H23" t="s">
-        <v>13</v>
-      </c>
-      <c r="I23" t="s">
-        <v>13</v>
-      </c>
-      <c r="L23" t="s">
-        <v>175</v>
-      </c>
-      <c r="M23" t="s">
-        <v>174</v>
-      </c>
-      <c r="N23" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B24" t="s">
-        <v>157</v>
-      </c>
-      <c r="F24" t="str">
-        <f t="shared" ref="F24:F27" si="8">L24</f>
-        <v>Mt-y</v>
-      </c>
-      <c r="G24" t="str">
-        <f t="shared" ref="G24:G26" si="9">M24&amp;" [TIMESreport "&amp;N24&amp;"]"</f>
-        <v>Million ton a year [TIMESreport capacityunit]</v>
-      </c>
-      <c r="H24" t="s">
-        <v>13</v>
-      </c>
-      <c r="I24" t="s">
-        <v>13</v>
-      </c>
-      <c r="L24" t="s">
-        <v>162</v>
-      </c>
-      <c r="M24" t="s">
-        <v>163</v>
-      </c>
-      <c r="N24" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>184</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="F25" t="str">
-        <f t="shared" si="8"/>
-        <v>PJa</v>
-      </c>
-      <c r="G25" t="str">
-        <f t="shared" si="9"/>
-        <v>PJ annually [TIMESreport capacityunit]</v>
-      </c>
-      <c r="H25" t="s">
-        <v>13</v>
-      </c>
-      <c r="I25" t="s">
-        <v>13</v>
-      </c>
-      <c r="L25" t="s">
-        <v>180</v>
-      </c>
-      <c r="M25" t="s">
-        <v>181</v>
-      </c>
-      <c r="N25" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>130</v>
-      </c>
-      <c r="F26" t="str">
-        <f t="shared" si="8"/>
-        <v>GW</v>
-      </c>
-      <c r="G26" t="str">
-        <f t="shared" si="9"/>
-        <v>GW [TIMESreport capacityunit]</v>
-      </c>
-      <c r="H26" t="s">
-        <v>13</v>
-      </c>
-      <c r="I26" t="s">
-        <v>13</v>
-      </c>
-      <c r="L26" t="s">
-        <v>182</v>
-      </c>
-      <c r="M26" t="s">
-        <v>182</v>
-      </c>
-      <c r="N26" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>138</v>
-      </c>
-      <c r="F27" t="str">
-        <f t="shared" si="8"/>
-        <v>000_Units</v>
-      </c>
-      <c r="G27" t="str">
-        <f t="shared" ref="G27" si="10">M27&amp;" [TIMESreport "&amp;N27&amp;"]"</f>
-        <v>1000 units [TIMESreport capacityunit]</v>
-      </c>
-      <c r="H27" t="s">
-        <v>13</v>
-      </c>
-      <c r="I27" t="s">
-        <v>13</v>
-      </c>
-      <c r="L27" t="s">
-        <v>185</v>
-      </c>
-      <c r="M27" t="s">
-        <v>186</v>
-      </c>
-      <c r="N27" t="s">
-        <v>179</v>
+        <v>Renewable [TIMESreport techgroup]</v>
+      </c>
+      <c r="H54" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="L54" t="s">
+        <v>13</v>
+      </c>
+      <c r="M54" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
+        <v>250</v>
+      </c>
+      <c r="B55" t="s">
+        <v>251</v>
+      </c>
+      <c r="C55" t="s">
+        <v>122</v>
+      </c>
+      <c r="E55" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_COA</v>
+      </c>
+      <c r="F55" t="str">
+        <f t="shared" si="5"/>
+        <v>Coal  [TIMESreport techgroup]</v>
+      </c>
+      <c r="H55" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J55" t="s">
+        <v>15</v>
+      </c>
+      <c r="L55" t="s">
+        <v>13</v>
+      </c>
+      <c r="M55" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="56" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
+        <v>266</v>
+      </c>
+      <c r="B56" t="s">
+        <v>267</v>
+      </c>
+      <c r="C56" t="s">
+        <v>122</v>
+      </c>
+      <c r="E56" t="str">
+        <f t="shared" si="4"/>
+        <v>TG_DMD</v>
+      </c>
+      <c r="F56" t="str">
+        <f t="shared" ref="F56" si="6">B56&amp;" [TIMESreport "&amp;C56&amp;"]"</f>
+        <v>Demand Technology [TIMESreport techgroup]</v>
+      </c>
+      <c r="H56" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="J56" t="s">
+        <v>15</v>
+      </c>
+      <c r="L56" t="s">
+        <v>13</v>
+      </c>
+      <c r="M56" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>